<commit_message>
Data computation over xlsx files
</commit_message>
<xml_diff>
--- a/data/raw/unused/BR_processed_time_calculations.xlsx
+++ b/data/raw/unused/BR_processed_time_calculations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jcastano-san\Documents\GitHub\E.Coli-model\data\raw\unused\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{97DE9C03-7A04-4CC4-A7F1-37B57F1BC8DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41645428-7E9C-45B9-919F-60DE4F8006B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38505" yWindow="-21855" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView minimized="1" xWindow="2655" yWindow="-13830" windowWidth="14340" windowHeight="8145" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -313,17 +313,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="21">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="6">
     <dxf>
       <font>
         <color rgb="FF9C5700"/>
@@ -371,146 +361,6 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C5700"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFEB9C"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1833,7 +1683,7 @@
         <v>3.2522952787326372E-2</v>
       </c>
       <c r="AH10">
-        <f>D10-D9</f>
+        <f t="shared" ref="AH10:AH18" si="0">D10-D9</f>
         <v>0.59999999999999787</v>
       </c>
       <c r="AN10">
@@ -1935,7 +1785,7 @@
         <v>0.10759104372641751</v>
       </c>
       <c r="AH11">
-        <f>D11-D10</f>
+        <f t="shared" si="0"/>
         <v>1.2833333333333314</v>
       </c>
       <c r="AN11">
@@ -2037,7 +1887,7 @@
         <v>8.9098470541607938E-2</v>
       </c>
       <c r="AH12">
-        <f>D12-D11</f>
+        <f t="shared" si="0"/>
         <v>1.7499999999999964</v>
       </c>
       <c r="AN12">
@@ -2139,7 +1989,7 @@
         <v>6.9185636517280089E-2</v>
       </c>
       <c r="AH13">
-        <f>D13-D12</f>
+        <f t="shared" si="0"/>
         <v>2.1166666666666707</v>
       </c>
       <c r="AN13">
@@ -2241,7 +2091,7 @@
         <v>0.1198064517436091</v>
       </c>
       <c r="AH14">
-        <f>D14-D13</f>
+        <f t="shared" si="0"/>
         <v>2</v>
       </c>
       <c r="AN14">
@@ -2343,7 +2193,7 @@
         <v>0.2433063684827845</v>
       </c>
       <c r="AH15">
-        <f>D15-D14</f>
+        <f t="shared" si="0"/>
         <v>1.9500000000000011</v>
       </c>
       <c r="AN15">
@@ -2445,7 +2295,7 @@
         <v>0.3596705739649278</v>
       </c>
       <c r="AH16">
-        <f>D16-D15</f>
+        <f t="shared" si="0"/>
         <v>1.0499999999999972</v>
       </c>
       <c r="AN16">
@@ -2547,7 +2397,7 @@
         <v>0.53870385406425392</v>
       </c>
       <c r="AH17">
-        <f>D17-D16</f>
+        <f t="shared" si="0"/>
         <v>1.0166666666666728</v>
       </c>
       <c r="AN17">
@@ -2649,7 +2499,7 @@
         <v>0.75148625307719852</v>
       </c>
       <c r="AH18">
-        <f>D18-D17</f>
+        <f t="shared" si="0"/>
         <v>0.96666666666666856</v>
       </c>
       <c r="AN18">
@@ -3767,7 +3617,7 @@
         <v>0.1003600680355974</v>
       </c>
       <c r="AH29">
-        <f t="shared" ref="AH29:AH36" si="0">D29-D28</f>
+        <f t="shared" ref="AH29:AH33" si="1">D29-D28</f>
         <v>1.75</v>
       </c>
       <c r="AN29">
@@ -3869,7 +3719,7 @@
         <v>5.1129804866170137E-3</v>
       </c>
       <c r="AH30">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2.1166666666666707</v>
       </c>
       <c r="AN30">
@@ -3971,7 +3821,7 @@
         <v>0.17511196653419439</v>
       </c>
       <c r="AH31">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>2</v>
       </c>
       <c r="AN31">
@@ -4073,7 +3923,7 @@
         <v>0.72407301857260176</v>
       </c>
       <c r="AH32">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1.93333333333333</v>
       </c>
       <c r="AN32">
@@ -4175,7 +4025,7 @@
         <v>1.133132459695009</v>
       </c>
       <c r="AH33">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1.06666666666667</v>
       </c>
       <c r="AN33">
@@ -4375,7 +4225,7 @@
         <v>0</v>
       </c>
       <c r="AF35">
-        <f>C35-C34</f>
+        <f t="shared" ref="AF35:AF41" si="2">C35-C34</f>
         <v>0.68333333333333357</v>
       </c>
       <c r="AN35">
@@ -4477,7 +4327,7 @@
         <v>0</v>
       </c>
       <c r="AF36">
-        <f>C36-C35</f>
+        <f t="shared" si="2"/>
         <v>1.0333333333333323</v>
       </c>
       <c r="AN36">
@@ -4579,7 +4429,7 @@
         <v>0</v>
       </c>
       <c r="AF37">
-        <f>C37-C36</f>
+        <f t="shared" si="2"/>
         <v>0.43333333333333224</v>
       </c>
       <c r="AN37">
@@ -4681,7 +4531,7 @@
         <v>0</v>
       </c>
       <c r="AF38">
-        <f>C38-C37</f>
+        <f t="shared" si="2"/>
         <v>0.51666666666666705</v>
       </c>
       <c r="AN38">
@@ -4783,7 +4633,7 @@
         <v>0</v>
       </c>
       <c r="AF39">
-        <f>C39-C38</f>
+        <f t="shared" si="2"/>
         <v>0.50000000000000089</v>
       </c>
       <c r="AN39">
@@ -4885,7 +4735,7 @@
         <v>0</v>
       </c>
       <c r="AF40">
-        <f>C40-C39</f>
+        <f t="shared" si="2"/>
         <v>0.49999999999999911</v>
       </c>
       <c r="AN40">
@@ -4987,7 +4837,7 @@
         <v>0</v>
       </c>
       <c r="AF41">
-        <f>C41-C40</f>
+        <f t="shared" si="2"/>
         <v>0.50000000000000178</v>
       </c>
       <c r="AN41">
@@ -5191,7 +5041,7 @@
         <v>0</v>
       </c>
       <c r="AG43">
-        <f t="shared" ref="AG43:AG48" si="1">C43-C42</f>
+        <f t="shared" ref="AG43:AG48" si="3">C43-C42</f>
         <v>0.90000000000000036</v>
       </c>
       <c r="AN43">
@@ -5293,7 +5143,7 @@
         <v>0</v>
       </c>
       <c r="AG44">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.95000000000000107</v>
       </c>
       <c r="AN44">
@@ -5395,7 +5245,7 @@
         <v>0</v>
       </c>
       <c r="AG45">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.50000000000000266</v>
       </c>
       <c r="AN45">
@@ -5497,7 +5347,7 @@
         <v>0</v>
       </c>
       <c r="AG46">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.71666666666666501</v>
       </c>
       <c r="AN46">
@@ -5599,7 +5449,7 @@
         <v>0</v>
       </c>
       <c r="AG47">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.63333333333333286</v>
       </c>
       <c r="AN47">
@@ -5701,7 +5551,7 @@
         <v>0</v>
       </c>
       <c r="AG48">
-        <f t="shared" si="1"/>
+        <f t="shared" si="3"/>
         <v>0.61666666666666714</v>
       </c>
       <c r="AN48">
@@ -5905,7 +5755,7 @@
         <v>4.345502810914946E-2</v>
       </c>
       <c r="AH50">
-        <f t="shared" ref="AH50:AH54" si="2">D50-D49</f>
+        <f t="shared" ref="AH50:AH54" si="4">D50-D49</f>
         <v>1.0999999999999979</v>
       </c>
       <c r="AN50">
@@ -6007,7 +5857,7 @@
         <v>2.8748570025759951E-2</v>
       </c>
       <c r="AH51">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.93333333333333002</v>
       </c>
       <c r="AN51">
@@ -6109,7 +5959,7 @@
         <v>4.5853213189522728E-2</v>
       </c>
       <c r="AH52">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1.0000000000000107</v>
       </c>
       <c r="AN52">
@@ -6211,7 +6061,7 @@
         <v>8.4628820173168973E-2</v>
       </c>
       <c r="AH53">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>1.0833333333333304</v>
       </c>
       <c r="AN53">
@@ -6313,7 +6163,7 @@
         <v>0.1139189019976181</v>
       </c>
       <c r="AH54">
-        <f t="shared" si="2"/>
+        <f t="shared" si="4"/>
         <v>0.88333333333332931</v>
       </c>
       <c r="AN54">
@@ -6513,7 +6363,7 @@
         <v>0</v>
       </c>
       <c r="AF56">
-        <f>C56-C55</f>
+        <f t="shared" ref="AF56:AF64" si="5">C56-C55</f>
         <v>0.68333333333333357</v>
       </c>
       <c r="AN56">
@@ -6615,7 +6465,7 @@
         <v>0</v>
       </c>
       <c r="AF57">
-        <f>C57-C56</f>
+        <f t="shared" si="5"/>
         <v>1.0333333333333323</v>
       </c>
       <c r="AN57">
@@ -6717,7 +6567,7 @@
         <v>0</v>
       </c>
       <c r="AF58">
-        <f>C58-C57</f>
+        <f t="shared" si="5"/>
         <v>0.43333333333333224</v>
       </c>
       <c r="AN58">
@@ -6819,7 +6669,7 @@
         <v>0</v>
       </c>
       <c r="AF59">
-        <f>C59-C58</f>
+        <f t="shared" si="5"/>
         <v>0.46666666666666679</v>
       </c>
       <c r="AN59">
@@ -6921,7 +6771,7 @@
         <v>0</v>
       </c>
       <c r="AF60">
-        <f>C60-C59</f>
+        <f t="shared" si="5"/>
         <v>0.55000000000000115</v>
       </c>
       <c r="AN60">
@@ -7023,7 +6873,7 @@
         <v>0</v>
       </c>
       <c r="AF61">
-        <f>C61-C60</f>
+        <f t="shared" si="5"/>
         <v>0.49999999999999911</v>
       </c>
       <c r="AN61">
@@ -7125,7 +6975,7 @@
         <v>0</v>
       </c>
       <c r="AF62">
-        <f>C62-C61</f>
+        <f t="shared" si="5"/>
         <v>0.50000000000000178</v>
       </c>
       <c r="AN62">
@@ -7227,7 +7077,7 @@
         <v>0</v>
       </c>
       <c r="AF63">
-        <f>C63-C62</f>
+        <f t="shared" si="5"/>
         <v>0.48333333333333073</v>
       </c>
       <c r="AN63">
@@ -7329,7 +7179,7 @@
         <v>0</v>
       </c>
       <c r="AF64">
-        <f>C64-C63</f>
+        <f t="shared" si="5"/>
         <v>0.8500000000000032</v>
       </c>
       <c r="AN64">
@@ -7431,7 +7281,7 @@
         <v>0</v>
       </c>
       <c r="AG65">
-        <f t="shared" ref="AG64:AG69" si="3">C65-C64</f>
+        <f t="shared" ref="AG65:AG69" si="6">C65-C64</f>
         <v>0.99999999999999822</v>
       </c>
       <c r="AN65">
@@ -7533,7 +7383,7 @@
         <v>0</v>
       </c>
       <c r="AG66">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>0.50000000000000266</v>
       </c>
       <c r="AN66">
@@ -7635,7 +7485,7 @@
         <v>0</v>
       </c>
       <c r="AG67">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>0.71666666666666501</v>
       </c>
       <c r="AN67">
@@ -7737,7 +7587,7 @@
         <v>0</v>
       </c>
       <c r="AG68">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>0.63333333333333286</v>
       </c>
       <c r="AN68">
@@ -7839,7 +7689,7 @@
         <v>0</v>
       </c>
       <c r="AG69">
-        <f t="shared" si="3"/>
+        <f t="shared" si="6"/>
         <v>0.71666666666666501</v>
       </c>
       <c r="AN69">
@@ -8043,7 +7893,7 @@
         <v>5.3631977825163497E-2</v>
       </c>
       <c r="AH71">
-        <f t="shared" ref="AH71:AH75" si="4">D71-D70</f>
+        <f t="shared" ref="AH71:AH75" si="7">D71-D70</f>
         <v>1.0999999999999979</v>
       </c>
       <c r="AN71">
@@ -8145,7 +7995,7 @@
         <v>4.1857480857527468E-2</v>
       </c>
       <c r="AH72">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v>0.96666666666667034</v>
       </c>
       <c r="AN72">
@@ -8247,7 +8097,7 @@
         <v>2.6686124435171231E-2</v>
       </c>
       <c r="AH73">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v>1</v>
       </c>
       <c r="AN73">
@@ -8349,7 +8199,7 @@
         <v>1.042051580594177E-2</v>
       </c>
       <c r="AH74">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v>1.0500000000000007</v>
       </c>
       <c r="AN74">
@@ -8451,7 +8301,7 @@
         <v>2.8120085825098141E-4</v>
       </c>
       <c r="AH75">
-        <f t="shared" si="4"/>
+        <f t="shared" si="7"/>
         <v>0.86666666666666892</v>
       </c>
       <c r="AN75">
@@ -9161,7 +9011,7 @@
         <v>0</v>
       </c>
       <c r="AG82">
-        <f t="shared" ref="AG78:AG84" si="5">C82-C81</f>
+        <f t="shared" ref="AG82:AG83" si="8">C82-C81</f>
         <v>0.95000000000000284</v>
       </c>
       <c r="AN82">
@@ -9263,7 +9113,7 @@
         <v>0</v>
       </c>
       <c r="AG83">
-        <f t="shared" si="5"/>
+        <f t="shared" si="8"/>
         <v>0.96666666666666501</v>
       </c>
       <c r="AN83">
@@ -9464,7 +9314,7 @@
         <v>0</v>
       </c>
       <c r="AG85">
-        <f t="shared" ref="AG85:AG90" si="6">C85-C84</f>
+        <f t="shared" ref="AG85:AG90" si="9">C85-C84</f>
         <v>1.2666666666666648</v>
       </c>
     </row>
@@ -9563,7 +9413,7 @@
         <v>0</v>
       </c>
       <c r="AG86">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>0.90000000000000302</v>
       </c>
     </row>
@@ -9662,7 +9512,7 @@
         <v>0</v>
       </c>
       <c r="AG87">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>1</v>
       </c>
     </row>
@@ -9761,7 +9611,7 @@
         <v>0</v>
       </c>
       <c r="AG88">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>1.1499999999999986</v>
       </c>
     </row>
@@ -9860,7 +9710,7 @@
         <v>0</v>
       </c>
       <c r="AG89">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>1.4166666666666696</v>
       </c>
     </row>
@@ -9959,7 +9809,7 @@
         <v>7.4129435761987661E-2</v>
       </c>
       <c r="AG90">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>0.8999999999999897</v>
       </c>
     </row>
@@ -10157,7 +10007,7 @@
         <v>4.9577837271181403E-2</v>
       </c>
       <c r="AH92">
-        <f t="shared" ref="AH92:AH102" si="7">D92-D91</f>
+        <f t="shared" ref="AH92:AH102" si="10">D92-D91</f>
         <v>1.5</v>
       </c>
     </row>
@@ -10256,7 +10106,7 @@
         <v>3.3314935299776048E-2</v>
       </c>
       <c r="AH93">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>2</v>
       </c>
     </row>
@@ -10355,7 +10205,7 @@
         <v>4.1506261929767606E-3</v>
       </c>
       <c r="AH94">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>4.3333333333333286</v>
       </c>
     </row>
@@ -10454,7 +10304,7 @@
         <v>1.1798492787110711E-3</v>
       </c>
       <c r="AH95">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>1.6666666666666714</v>
       </c>
     </row>
@@ -10553,7 +10403,7 @@
         <v>1.2503461527181121E-3</v>
       </c>
       <c r="AH96">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>2.5</v>
       </c>
     </row>
@@ -10751,7 +10601,7 @@
         <v>1.2793703302239651E-3</v>
       </c>
       <c r="AH98">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>2.7833333333333385</v>
       </c>
     </row>
@@ -10850,7 +10700,7 @@
         <v>1.31211416093447E-3</v>
       </c>
       <c r="AH99">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>3.0500000000000007</v>
       </c>
     </row>
@@ -10949,7 +10799,7 @@
         <v>9.2909463277215457E-3</v>
       </c>
       <c r="AH100">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>3</v>
       </c>
     </row>
@@ -11048,7 +10898,7 @@
         <v>2.1765796615230881E-2</v>
       </c>
       <c r="AH101">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>2.5833333333333428</v>
       </c>
     </row>
@@ -11149,7 +10999,7 @@
       <c r="AF102" s="6"/>
       <c r="AG102" s="6"/>
       <c r="AH102" s="7">
-        <f t="shared" si="7"/>
+        <f t="shared" si="10"/>
         <v>7.5999999999999943</v>
       </c>
     </row>
@@ -11640,7 +11490,7 @@
         <v>0</v>
       </c>
       <c r="AG107">
-        <f t="shared" ref="AG105:AG111" si="8">C107-C106</f>
+        <f t="shared" ref="AG107:AG110" si="11">C107-C106</f>
         <v>0.96666666666666767</v>
       </c>
     </row>
@@ -11739,7 +11589,7 @@
         <v>0</v>
       </c>
       <c r="AG108">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>0.96666666666666501</v>
       </c>
     </row>
@@ -11838,7 +11688,7 @@
         <v>0</v>
       </c>
       <c r="AG109">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>0.86666666666666714</v>
       </c>
     </row>
@@ -11937,7 +11787,7 @@
         <v>0</v>
       </c>
       <c r="AG110">
-        <f t="shared" si="8"/>
+        <f t="shared" si="11"/>
         <v>1.0833333333333339</v>
       </c>
     </row>
@@ -12135,7 +11985,7 @@
         <v>0</v>
       </c>
       <c r="AG112">
-        <f t="shared" ref="AG112:AG116" si="9">C112-C111</f>
+        <f t="shared" ref="AG112:AG116" si="12">C112-C111</f>
         <v>0.61666666666666625</v>
       </c>
     </row>
@@ -12234,7 +12084,7 @@
         <v>0</v>
       </c>
       <c r="AG113">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>0.80000000000000071</v>
       </c>
     </row>
@@ -12333,7 +12183,7 @@
         <v>4.3066416552685567E-2</v>
       </c>
       <c r="AG114">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>1.0833333333333286</v>
       </c>
     </row>
@@ -12432,7 +12282,7 @@
         <v>3.7890617921065912E-2</v>
       </c>
       <c r="AG115">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>1.4333333333333407</v>
       </c>
     </row>
@@ -12531,7 +12381,7 @@
         <v>3.3727497888753573E-2</v>
       </c>
       <c r="AG116">
-        <f t="shared" si="9"/>
+        <f t="shared" si="12"/>
         <v>1.0999999999999996</v>
       </c>
     </row>
@@ -12729,7 +12579,7 @@
         <v>1.63849784521229E-2</v>
       </c>
       <c r="AH118">
-        <f t="shared" ref="AH118:AH124" si="10">D118-D117</f>
+        <f t="shared" ref="AH118:AH123" si="13">D118-D117</f>
         <v>2.7166666666666721</v>
       </c>
     </row>
@@ -12828,7 +12678,7 @@
         <v>4.9368558210821792E-3</v>
       </c>
       <c r="AH119">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>5.5499999999999972</v>
       </c>
     </row>
@@ -12927,7 +12777,7 @@
         <v>3.7766365160811911E-3</v>
       </c>
       <c r="AH120">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>1.6500000000000021</v>
       </c>
     </row>
@@ -13026,7 +12876,7 @@
         <v>3.7778124103728218E-3</v>
       </c>
       <c r="AH121">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>1.5</v>
       </c>
     </row>
@@ -13125,7 +12975,7 @@
         <v>4.344176341084042E-3</v>
       </c>
       <c r="AH122">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>1.4666666666666686</v>
       </c>
     </row>
@@ -13224,7 +13074,7 @@
         <v>7.5847434595864398E-3</v>
       </c>
       <c r="AH123">
-        <f t="shared" si="10"/>
+        <f t="shared" si="13"/>
         <v>3.0333333333333314</v>
       </c>
     </row>
@@ -14158,7 +14008,7 @@
         <v>0</v>
       </c>
       <c r="AG132">
-        <f t="shared" ref="AG130:AG136" si="11">C132-C131</f>
+        <f t="shared" ref="AG132:AG135" si="14">C132-C131</f>
         <v>1.2166666666666659</v>
       </c>
       <c r="AL132" t="s">
@@ -14263,7 +14113,7 @@
         <v>0</v>
       </c>
       <c r="AG133">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>0.96666666666666856</v>
       </c>
       <c r="AK133" t="s">
@@ -14373,7 +14223,7 @@
         <v>0</v>
       </c>
       <c r="AG134">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>0.99999999999999822</v>
       </c>
     </row>
@@ -14472,7 +14322,7 @@
         <v>0</v>
       </c>
       <c r="AG135">
-        <f t="shared" si="11"/>
+        <f t="shared" si="14"/>
         <v>0.86666666666666714</v>
       </c>
     </row>
@@ -14913,7 +14763,7 @@
         <v>0</v>
       </c>
       <c r="AH139">
-        <f t="shared" ref="AH139:AH145" si="12">D139-D138</f>
+        <f t="shared" ref="AH139:AH144" si="15">D139-D138</f>
         <v>0.73333333333333073</v>
       </c>
       <c r="AL139" t="s">
@@ -15018,7 +14868,7 @@
         <v>0</v>
       </c>
       <c r="AH140">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>1.1166666666666689</v>
       </c>
       <c r="AK140" t="s">
@@ -15128,7 +14978,7 @@
         <v>0</v>
       </c>
       <c r="AH141">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>1.4666666666666703</v>
       </c>
     </row>
@@ -15227,7 +15077,7 @@
         <v>0</v>
       </c>
       <c r="AH142">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>1.18333333333333</v>
       </c>
     </row>
@@ -15326,7 +15176,7 @@
         <v>0</v>
       </c>
       <c r="AH143">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>1.4666666666666703</v>
       </c>
       <c r="AK143" t="s">
@@ -15434,7 +15284,7 @@
         <v>0</v>
       </c>
       <c r="AH144">
-        <f t="shared" si="12"/>
+        <f t="shared" si="15"/>
         <v>2.6666666666666607</v>
       </c>
       <c r="AK144" t="s">
@@ -15675,7 +15525,7 @@
         <v>0</v>
       </c>
       <c r="AH146">
-        <f t="shared" ref="AH146:AH152" si="13">D146-D145</f>
+        <f t="shared" ref="AH146:AH152" si="16">D146-D145</f>
         <v>1.5666666666666593</v>
       </c>
       <c r="AL146" t="s">
@@ -15780,7 +15630,7 @@
         <v>0</v>
       </c>
       <c r="AH147">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>1.5500000000000007</v>
       </c>
       <c r="AK147" t="s">
@@ -15894,7 +15744,7 @@
         <v>0</v>
       </c>
       <c r="AH148">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>1.4666666666666686</v>
       </c>
       <c r="AQ148">
@@ -15997,7 +15847,7 @@
         <v>0</v>
       </c>
       <c r="AH149">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>3.0333333333333314</v>
       </c>
     </row>
@@ -16096,7 +15946,7 @@
         <v>0</v>
       </c>
       <c r="AH150">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>3.0000000000000071</v>
       </c>
     </row>
@@ -16195,7 +16045,7 @@
         <v>0</v>
       </c>
       <c r="AH151">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>1.5166666666666657</v>
       </c>
     </row>
@@ -16294,7 +16144,7 @@
         <v>0</v>
       </c>
       <c r="AH152">
-        <f t="shared" si="13"/>
+        <f t="shared" si="16"/>
         <v>1.0499999999999972</v>
       </c>
     </row>
@@ -16518,28 +16368,28 @@
     <sortCondition descending="1" ref="AN3:AN173"/>
   </sortState>
   <conditionalFormatting sqref="AF3:AF159">
-    <cfRule type="cellIs" dxfId="10" priority="6" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="5" priority="6" operator="greaterThan">
       <formula>$AN$131</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="5" operator="between">
+    <cfRule type="cellIs" dxfId="4" priority="5" operator="between">
       <formula>0.001</formula>
       <formula>$AO$131</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AG6:AG164">
-    <cfRule type="cellIs" dxfId="8" priority="4" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="3" priority="4" operator="greaterThan">
       <formula>$AN$138</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="3" operator="between">
+    <cfRule type="cellIs" dxfId="2" priority="3" operator="between">
       <formula>0.00001</formula>
       <formula>$AO$138</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AH10:AH180">
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="greaterThan">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="greaterThan">
       <formula>$AN$145</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="between">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="between">
       <formula>0.0001</formula>
       <formula>$AO$145</formula>
     </cfRule>

</xml_diff>